<commit_message>
docs: estado del Sprint 4 y validacion de empresas en el Sprint 5
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/cronograma.xlsx
+++ b/docs/cronograma.xlsx
@@ -188,10 +188,10 @@
     <t>31 oct – 6 nov</t>
   </si>
   <si>
-    <t>Módulo empresarial, búsqueda y consulta de perfiles</t>
-  </si>
-  <si>
-    <t>Módulo empresarial</t>
+    <t>Módulo empresarial, búsqueda y consulta de perfiles, y validación de empresas (rol Validador de Empresas)</t>
+  </si>
+  <si>
+    <t>Módulo empresarial + validación de empresas</t>
   </si>
   <si>
     <t>10. Integración general</t>

</xml_diff>